<commit_message>
update data indicators to June and adjust filters
</commit_message>
<xml_diff>
--- a/Espelho_Indicadores_BSC.xlsx
+++ b/Espelho_Indicadores_BSC.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="129">
   <si>
     <t>Operação</t>
   </si>
@@ -22,7 +22,7 @@
     <t>Meta 4 Pontos</t>
   </si>
   <si>
-    <t>Mai</t>
+    <t>Jun</t>
   </si>
   <si>
     <t>W22</t>
@@ -52,112 +52,133 @@
     <t>97.9%</t>
   </si>
   <si>
-    <t>96.75 %</t>
+    <t>96.85 %</t>
+  </si>
+  <si>
+    <t>97.91 %</t>
+  </si>
+  <si>
+    <t>95.65 %</t>
+  </si>
+  <si>
+    <t>96.4 %</t>
+  </si>
+  <si>
+    <t>97.3 %</t>
+  </si>
+  <si>
+    <t>97.69 %</t>
+  </si>
+  <si>
+    <t>97.86 %</t>
+  </si>
+  <si>
+    <t>Pickup Sucess (Ontime) FULL</t>
+  </si>
+  <si>
+    <t>92.6%</t>
+  </si>
+  <si>
+    <t>91.75 %</t>
+  </si>
+  <si>
+    <t>92.02 %</t>
+  </si>
+  <si>
+    <t>89.53 %</t>
+  </si>
+  <si>
+    <t>88.75 %</t>
+  </si>
+  <si>
+    <t>93.37 %</t>
+  </si>
+  <si>
+    <t>94.82 %</t>
+  </si>
+  <si>
+    <t>94.29 %</t>
+  </si>
+  <si>
+    <t>Aderência ao Perfil FULL</t>
+  </si>
+  <si>
+    <t>95%</t>
+  </si>
+  <si>
+    <t>94.4 %</t>
+  </si>
+  <si>
+    <t>98.47 %</t>
+  </si>
+  <si>
+    <t>94.7 %</t>
+  </si>
+  <si>
+    <t>97.87 %</t>
+  </si>
+  <si>
+    <t>96.17 %</t>
+  </si>
+  <si>
+    <t>96.79 %</t>
+  </si>
+  <si>
+    <t>% Utilização Frota Fixa FULL</t>
+  </si>
+  <si>
+    <t>86.68 %</t>
+  </si>
+  <si>
+    <t>87.38 %</t>
+  </si>
+  <si>
+    <t>89.46 %</t>
+  </si>
+  <si>
+    <t>84.79 %</t>
+  </si>
+  <si>
+    <t>84.96 %</t>
+  </si>
+  <si>
+    <t>85.83 %</t>
+  </si>
+  <si>
+    <t>82.54 %</t>
+  </si>
+  <si>
+    <t>Aceite de Scheduling XD</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>95.65 %</t>
-  </si>
-  <si>
-    <t>96.4 %</t>
-  </si>
-  <si>
-    <t>97.3 %</t>
-  </si>
-  <si>
-    <t>97.67 %</t>
-  </si>
-  <si>
-    <t>87.54 %</t>
-  </si>
-  <si>
-    <t>Pickup Sucess (Ontime) FULL</t>
-  </si>
-  <si>
-    <t>92.6%</t>
-  </si>
-  <si>
-    <t>92.12 %</t>
-  </si>
-  <si>
-    <t>89.53 %</t>
-  </si>
-  <si>
-    <t>88.75 %</t>
-  </si>
-  <si>
-    <t>93.37 %</t>
-  </si>
-  <si>
-    <t>94.77 %</t>
-  </si>
-  <si>
-    <t>84.13 %</t>
-  </si>
-  <si>
-    <t>Aderência ao Perfil FULL</t>
-  </si>
-  <si>
-    <t>95%</t>
-  </si>
-  <si>
-    <t>94.78 %</t>
-  </si>
-  <si>
-    <t>98.47 %</t>
-  </si>
-  <si>
-    <t>94.7 %</t>
-  </si>
-  <si>
-    <t>97.87 %</t>
-  </si>
-  <si>
-    <t>96.53 %</t>
-  </si>
-  <si>
-    <t>99.36 %</t>
-  </si>
-  <si>
-    <t>% Utilização Frota Fixa FULL</t>
-  </si>
-  <si>
-    <t>83.69 %</t>
-  </si>
-  <si>
-    <t>89.46 %</t>
-  </si>
-  <si>
-    <t>84.79 %</t>
-  </si>
-  <si>
-    <t>84.96 %</t>
-  </si>
-  <si>
-    <t>85.83 %</t>
-  </si>
-  <si>
-    <t>58.44 %</t>
-  </si>
-  <si>
-    <t>Aceite de Scheduling XD</t>
-  </si>
-  <si>
     <t>Ad. Config XD</t>
   </si>
   <si>
     <t>97%</t>
   </si>
   <si>
-    <t>96.47 %</t>
-  </si>
-  <si>
-    <t>107.85 %</t>
-  </si>
-  <si>
-    <t>3012.14 %</t>
+    <t>96.22 %</t>
+  </si>
+  <si>
+    <t>101.24 %</t>
+  </si>
+  <si>
+    <t>99.94 %</t>
+  </si>
+  <si>
+    <t>99.79 %</t>
+  </si>
+  <si>
+    <t>99.75 %</t>
+  </si>
+  <si>
+    <t>84.69 %</t>
+  </si>
+  <si>
+    <t>99.6 %</t>
   </si>
   <si>
     <t>Last Mile</t>
@@ -169,7 +190,10 @@
     <t>98.2%</t>
   </si>
   <si>
-    <t>96.08 %</t>
+    <t>96.04 %</t>
+  </si>
+  <si>
+    <t>96.05 %</t>
   </si>
   <si>
     <t>96.11 %</t>
@@ -181,97 +205,109 @@
     <t>95.75 %</t>
   </si>
   <si>
+    <t>96.24 %</t>
+  </si>
+  <si>
+    <t>% Real x D7 FDS (SVC) SPOT</t>
+  </si>
+  <si>
+    <t>90%</t>
+  </si>
+  <si>
+    <t>69.23 %</t>
+  </si>
+  <si>
+    <t>63.64 %</t>
+  </si>
+  <si>
+    <t>54.55 %</t>
+  </si>
+  <si>
+    <t>66.67 %</t>
+  </si>
+  <si>
+    <t>58.33 %</t>
+  </si>
+  <si>
+    <t>75 %</t>
+  </si>
+  <si>
+    <t>Aceite Scheduling Pré Routing</t>
+  </si>
+  <si>
+    <t>5%</t>
+  </si>
+  <si>
+    <t>3.99 %</t>
+  </si>
+  <si>
+    <t>6.13 %</t>
+  </si>
+  <si>
+    <t>5.03 %</t>
+  </si>
+  <si>
+    <t>3.78 %</t>
+  </si>
+  <si>
+    <t>4.14 %</t>
+  </si>
+  <si>
+    <t>3.95 %</t>
+  </si>
+  <si>
+    <t>1.61 %</t>
+  </si>
+  <si>
+    <t>SDD - % ER</t>
+  </si>
+  <si>
+    <t>90.46 %</t>
+  </si>
+  <si>
+    <t>82.41 %</t>
+  </si>
+  <si>
+    <t>91.83 %</t>
+  </si>
+  <si>
+    <t>95.76 %</t>
+  </si>
+  <si>
+    <t>89.78 %</t>
+  </si>
+  <si>
+    <t>86.82 %</t>
+  </si>
+  <si>
+    <t>87.83 %</t>
+  </si>
+  <si>
+    <t>% Utilização Frota Fixa (LM)</t>
+  </si>
+  <si>
+    <t>Delivery Success XPT</t>
+  </si>
+  <si>
+    <t>94.99 %</t>
+  </si>
+  <si>
+    <t>95.73 %</t>
+  </si>
+  <si>
+    <t>95.13 %</t>
+  </si>
+  <si>
+    <t>95.22 %</t>
+  </si>
+  <si>
     <t>94.75 %</t>
   </si>
   <si>
-    <t>% Real x D7 FDS (SVC) SPOT</t>
-  </si>
-  <si>
-    <t>90%</t>
-  </si>
-  <si>
-    <t>64.29 %</t>
-  </si>
-  <si>
-    <t>54.55 %</t>
-  </si>
-  <si>
-    <t>66.67 %</t>
-  </si>
-  <si>
-    <t>58.33 %</t>
-  </si>
-  <si>
-    <t>75 %</t>
-  </si>
-  <si>
-    <t>9.09 %</t>
-  </si>
-  <si>
-    <t>Aceite Scheduling Pré Routing</t>
-  </si>
-  <si>
-    <t>5%</t>
-  </si>
-  <si>
-    <t>5.74 %</t>
-  </si>
-  <si>
-    <t>5.03 %</t>
-  </si>
-  <si>
-    <t>3.78 %</t>
-  </si>
-  <si>
-    <t>4.14 %</t>
-  </si>
-  <si>
-    <t>3.95 %</t>
-  </si>
-  <si>
-    <t>1.91 %</t>
-  </si>
-  <si>
-    <t>SDD - % ER</t>
-  </si>
-  <si>
-    <t>73.61 %</t>
-  </si>
-  <si>
-    <t>91.83 %</t>
-  </si>
-  <si>
-    <t>95.76 %</t>
-  </si>
-  <si>
-    <t>89.78 %</t>
-  </si>
-  <si>
-    <t>87.5 %</t>
-  </si>
-  <si>
-    <t>0 %</t>
-  </si>
-  <si>
-    <t>% Utilização Frota Fixa (LM)</t>
-  </si>
-  <si>
-    <t>Delivery Success XPT</t>
-  </si>
-  <si>
-    <t>95.21 %</t>
-  </si>
-  <si>
-    <t>95.13 %</t>
-  </si>
-  <si>
-    <t>95.22 %</t>
-  </si>
-  <si>
     <t>95.01 %</t>
   </si>
   <si>
-    <t>87.92 %</t>
+    <t>94.54 %</t>
   </si>
   <si>
     <t>% Real x D7 FDS (XPT) SPOT</t>
@@ -292,16 +328,25 @@
     <t>72%</t>
   </si>
   <si>
-    <t>67.31 %</t>
-  </si>
-  <si>
-    <t>72.2 %</t>
-  </si>
-  <si>
-    <t>54.35 %</t>
-  </si>
-  <si>
-    <t>58.38 %</t>
+    <t>64.5 %</t>
+  </si>
+  <si>
+    <t>70.23 %</t>
+  </si>
+  <si>
+    <t>70.54 %</t>
+  </si>
+  <si>
+    <t>58.91 %</t>
+  </si>
+  <si>
+    <t>61.11 %</t>
+  </si>
+  <si>
+    <t>63.55 %</t>
+  </si>
+  <si>
+    <t>68.38 %</t>
   </si>
   <si>
     <t>Safety</t>
@@ -316,16 +361,31 @@
     <t>Telemetria Scorecard</t>
   </si>
   <si>
-    <t>78.4 %</t>
-  </si>
-  <si>
-    <t>77.44 %</t>
+    <t>78.6 %</t>
+  </si>
+  <si>
+    <t>89.77 %</t>
+  </si>
+  <si>
+    <t>84.01 %</t>
+  </si>
+  <si>
+    <t>88.17 %</t>
+  </si>
+  <si>
+    <t>81.32 %</t>
+  </si>
+  <si>
+    <t>87.47 %</t>
   </si>
   <si>
     <t>Aderência Treinamentos Safety Driver</t>
   </si>
   <si>
-    <t>96.8 %</t>
+    <t>96.41 %</t>
+  </si>
+  <si>
+    <t>97.31 %</t>
   </si>
   <si>
     <t>96.31 %</t>
@@ -337,7 +397,7 @@
     <t>96.23 %</t>
   </si>
   <si>
-    <t>96.76 %</t>
+    <t>96.83 %</t>
   </si>
 </sst>
 </file>
@@ -811,22 +871,22 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -834,31 +894,31 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -866,31 +926,31 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -898,31 +958,31 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -930,383 +990,383 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="J7" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="G8" t="s">
         <v>16</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="J8" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="G9" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="J9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="E10" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="F10" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="I10" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="J10" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="F11" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G11" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H11" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="I11" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="J11" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="F13" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="H13" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="J13" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="E14" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="F14" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="G14" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="I14" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="J14" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="E15" t="s">
-        <v>14</v>
+        <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H15" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="I15" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="J15" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="G16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="H16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="J16" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G17" t="s">
-        <v>14</v>
+        <v>118</v>
       </c>
       <c r="H17" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="I17" t="s">
-        <v>14</v>
+        <v>120</v>
       </c>
       <c r="J17" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="E18" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
       <c r="F18" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G18" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="H18" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="I18" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="J18" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add June weeks (W24, W25) to dashboard, mirror, and executive Excel generator
</commit_message>
<xml_diff>
--- a/Espelho_Indicadores_BSC.xlsx
+++ b/Espelho_Indicadores_BSC.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="127">
   <si>
     <t>Operação</t>
   </si>
@@ -25,6 +25,12 @@
     <t>Jun</t>
   </si>
   <si>
+    <t>W24</t>
+  </si>
+  <si>
+    <t>W25</t>
+  </si>
+  <si>
     <t>W26</t>
   </si>
   <si>
@@ -49,6 +55,12 @@
     <t>96.85 %</t>
   </si>
   <si>
+    <t>96.4 %</t>
+  </si>
+  <si>
+    <t>97.3 %</t>
+  </si>
+  <si>
     <t>97.69 %</t>
   </si>
   <si>
@@ -70,6 +82,12 @@
     <t>91.75 %</t>
   </si>
   <si>
+    <t>88.75 %</t>
+  </si>
+  <si>
+    <t>93.37 %</t>
+  </si>
+  <si>
     <t>94.82 %</t>
   </si>
   <si>
@@ -88,6 +106,12 @@
     <t>95%</t>
   </si>
   <si>
+    <t>94.7 %</t>
+  </si>
+  <si>
+    <t>97.87 %</t>
+  </si>
+  <si>
     <t>96.17 %</t>
   </si>
   <si>
@@ -106,15 +130,18 @@
     <t>86.68 %</t>
   </si>
   <si>
+    <t>84.79 %</t>
+  </si>
+  <si>
+    <t>84.96 %</t>
+  </si>
+  <si>
     <t>85.83 %</t>
   </si>
   <si>
     <t>82.54 %</t>
   </si>
   <si>
-    <t>84.96 %</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -130,6 +157,12 @@
     <t>96.22 %</t>
   </si>
   <si>
+    <t>99.79 %</t>
+  </si>
+  <si>
+    <t>99.75 %</t>
+  </si>
+  <si>
     <t>84.69 %</t>
   </si>
   <si>
@@ -154,6 +187,9 @@
     <t>96.04 %</t>
   </si>
   <si>
+    <t>96.07 %</t>
+  </si>
+  <si>
     <t>95.75 %</t>
   </si>
   <si>
@@ -175,6 +211,12 @@
     <t>69.23 %</t>
   </si>
   <si>
+    <t>66.67 %</t>
+  </si>
+  <si>
+    <t>58.33 %</t>
+  </si>
+  <si>
     <t>75 %</t>
   </si>
   <si>
@@ -196,6 +238,12 @@
     <t>3.99 %</t>
   </si>
   <si>
+    <t>3.78 %</t>
+  </si>
+  <si>
+    <t>4.14 %</t>
+  </si>
+  <si>
     <t>3.95 %</t>
   </si>
   <si>
@@ -214,6 +262,12 @@
     <t>90.46 %</t>
   </si>
   <si>
+    <t>95.76 %</t>
+  </si>
+  <si>
+    <t>89.78 %</t>
+  </si>
+  <si>
     <t>86.82 %</t>
   </si>
   <si>
@@ -238,6 +292,12 @@
     <t>94.99 %</t>
   </si>
   <si>
+    <t>95.22 %</t>
+  </si>
+  <si>
+    <t>94.75 %</t>
+  </si>
+  <si>
     <t>95.01 %</t>
   </si>
   <si>
@@ -256,6 +316,9 @@
     <t>80 %</t>
   </si>
   <si>
+    <t>100 %</t>
+  </si>
+  <si>
     <t>40 %</t>
   </si>
   <si>
@@ -268,6 +331,12 @@
     <t>64.5 %</t>
   </si>
   <si>
+    <t>58.91 %</t>
+  </si>
+  <si>
+    <t>61.11 %</t>
+  </si>
+  <si>
     <t>63.55 %</t>
   </si>
   <si>
@@ -289,6 +358,12 @@
     <t>Telemetria Scorecard</t>
   </si>
   <si>
+    <t>84.01 %</t>
+  </si>
+  <si>
+    <t>88.17 %</t>
+  </si>
+  <si>
     <t>81.32 %</t>
   </si>
   <si>
@@ -299,6 +374,12 @@
   </si>
   <si>
     <t>96.41 %</t>
+  </si>
+  <si>
+    <t>96.31 %</t>
+  </si>
+  <si>
+    <t>95.17 %</t>
   </si>
   <si>
     <t>96.23 %</t>
@@ -697,16 +778,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="8" width="10" customWidth="1"/>
+    <col min="4" max="10" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,447 +812,555 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="F8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" t="s">
+        <v>60</v>
+      </c>
+      <c r="I8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" t="s">
+        <v>77</v>
+      </c>
+      <c r="H10" t="s">
+        <v>78</v>
+      </c>
+      <c r="I10" t="s">
+        <v>79</v>
+      </c>
+      <c r="J10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" t="s">
         <v>30</v>
       </c>
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="D11" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" t="s">
+        <v>87</v>
+      </c>
+      <c r="J11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E12" t="s">
         <v>39</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F12" t="s">
         <v>40</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G12" t="s">
         <v>41</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H12" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="I12" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F13" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" t="s">
+        <v>96</v>
+      </c>
+      <c r="I13" t="s">
+        <v>97</v>
+      </c>
+      <c r="J13" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I14" t="s">
+        <v>102</v>
+      </c>
+      <c r="J14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" t="s">
+        <v>109</v>
+      </c>
+      <c r="I15" t="s">
+        <v>110</v>
+      </c>
+      <c r="J15" t="s">
         <v>43</v>
       </c>
-      <c r="B8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" t="s">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>113</v>
+      </c>
+      <c r="E16" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16" t="s">
+        <v>113</v>
+      </c>
+      <c r="H16" t="s">
+        <v>113</v>
+      </c>
+      <c r="I16" t="s">
+        <v>43</v>
+      </c>
+      <c r="J16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" t="s">
+        <v>117</v>
+      </c>
+      <c r="H17" t="s">
+        <v>118</v>
+      </c>
+      <c r="I17" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
         <v>46</v>
       </c>
-      <c r="E8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F11" t="s">
-        <v>68</v>
-      </c>
-      <c r="G11" t="s">
-        <v>69</v>
-      </c>
-      <c r="H11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>33</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E13" t="s">
-        <v>75</v>
-      </c>
-      <c r="F13" t="s">
-        <v>76</v>
-      </c>
-      <c r="G13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" t="s">
-        <v>81</v>
-      </c>
-      <c r="H14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" t="s">
-        <v>87</v>
-      </c>
-      <c r="H15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" t="s">
-        <v>90</v>
-      </c>
-      <c r="F16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" t="s">
-        <v>34</v>
-      </c>
-      <c r="H16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>88</v>
-      </c>
-      <c r="B17" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" t="s">
-        <v>92</v>
-      </c>
-      <c r="F17" t="s">
-        <v>93</v>
-      </c>
-      <c r="G17" t="s">
-        <v>34</v>
-      </c>
-      <c r="H17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" t="s">
-        <v>37</v>
-      </c>
       <c r="D18" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="F18" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="G18" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="H18" t="s">
-        <v>99</v>
+        <v>124</v>
+      </c>
+      <c r="I18" t="s">
+        <v>125</v>
+      </c>
+      <c r="J18" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>